<commit_message>
mml fix rolate doorprize
</commit_message>
<xml_diff>
--- a/MPMDOORPRIZE/MPMWEBDOORPRIZE/Scripts/templatehadiahdoorprize.xlsx
+++ b/MPMDOORPRIZE/MPMWEBDOORPRIZE/Scripts/templatehadiahdoorprize.xlsx
@@ -76,7 +76,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -360,15 +360,14 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="1"/>
-    <col min="3" max="5" width="8.7265625" style="1"/>
+    <col min="1" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">

</xml_diff>